<commit_message>
10/04/2026: Recipe module  test script completed
</commit_message>
<xml_diff>
--- a/com.SmartGatePuls.SDET/Automation.xlsx
+++ b/com.SmartGatePuls.SDET/Automation.xlsx
@@ -1,42 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Seleniumwebdriver\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEF0A03D-CC89-4E52-BB44-EB47E88E70EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{5C3FE741-22FA-4E87-8DFB-400CC1C71B4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="38640" windowHeight="15720" xr2:uid="{6452F18F-7895-4B2D-8A43-7E46840F2AF0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="0"/>
+  <oleSize ref="A1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="8">
   <si>
     <t>DeprtmentGroupName</t>
   </si>
@@ -47,9 +32,6 @@
     <t>DepartmentsName</t>
   </si>
   <si>
-    <t>AutomatonTest</t>
-  </si>
-  <si>
     <t>ReasonName</t>
   </si>
   <si>
@@ -57,6 +39,12 @@
   </si>
   <si>
     <t>AutomationReasonTestEdit</t>
+  </si>
+  <si>
+    <t>AutomationTest</t>
+  </si>
+  <si>
+    <t>RecipeAutomation</t>
   </si>
 </sst>
 </file>
@@ -428,7 +416,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3D5162B0-3621-417E-80E6-F58D97FFD320}">
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="21.6640625" customWidth="1"/>
@@ -436,7 +424,7 @@
     <col min="3" max="3" width="26.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -444,23 +432,29 @@
         <v>2</v>
       </c>
       <c r="C1" t="s">
-        <v>4</v>
+        <v>3</v>
+      </c>
+      <c r="D1" t="s">
+        <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="C2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C3" t="s">
         <v>5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="C3" t="s">
-        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
19/06/2026: User create modules script completed
</commit_message>
<xml_diff>
--- a/com.SmartGatePuls.SDET/Automation.xlsx
+++ b/com.SmartGatePuls.SDET/Automation.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{5C3FE741-22FA-4E87-8DFB-400CC1C71B4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{32C68012-B4ED-4984-8D32-BDC8E0FCE484}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="38640" windowHeight="15720" xr2:uid="{6452F18F-7895-4B2D-8A43-7E46840F2AF0}"/>
   </bookViews>
@@ -15,6 +15,9 @@
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="2"/>
     </ext>
   </extLst>
 </workbook>
@@ -453,6 +456,9 @@
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>123</v>
+      </c>
       <c r="C3" t="s">
         <v>5</v>
       </c>

</xml_diff>